<commit_message>
Update baseline models and run sheets for bergambacht_v2, eemdijk, ijkdijk, pernio
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/baseline_models/ijkdijk_runs.xlsx
+++ b/baseline_models/ijkdijk_runs.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28755" yWindow="-17985" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="runs" sheetId="1" state="visible" r:id="rId1"/>
@@ -3811,7 +3811,7 @@
         <v>10.5</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>0.76</v>
+        <v>0.26</v>
       </c>
       <c r="J5" s="12" t="n">
         <v>0.8</v>
@@ -3865,7 +3865,7 @@
         <v>10.5</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>0.76</v>
+        <v>0.26</v>
       </c>
       <c r="J6" s="14" t="n">
         <v>0.8</v>
@@ -3932,14 +3932,14 @@
           <t>0.0.0</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Sand_liquefiable</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>7_sand_liq</t>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>sand_pleistocene</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>6_Pleictoceen_zand</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -3952,21 +3952,23 @@
           <t>L 20</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>MohrCoulombClassic</t>
         </is>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="K8" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="18" t="n">
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="16" t="n">
+        <v>37.56</v>
+      </c>
+      <c r="L8" s="16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4076,7 +4078,7 @@
       </c>
       <c r="F11" s="32" t="inlineStr">
         <is>
-          <t>SuTable</t>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G11" s="30" t="n">
@@ -4115,7 +4117,7 @@
       </c>
       <c r="F12" s="32" t="inlineStr">
         <is>
-          <t>SuTable</t>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G12" s="30" t="n">
@@ -4154,7 +4156,7 @@
       </c>
       <c r="F13" s="32" t="inlineStr">
         <is>
-          <t>SuTable</t>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G13" s="30" t="n">
@@ -4193,7 +4195,7 @@
       </c>
       <c r="F14" s="32" t="inlineStr">
         <is>
-          <t>SuTable</t>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G14" s="30" t="n">
@@ -7444,9 +7446,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F77" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F77" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
@@ -7800,9 +7802,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F84" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F84" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G84" s="6" t="n">
@@ -8156,9 +8158,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F91" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F91" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G91" s="6" t="n">
@@ -8512,9 +8514,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F98" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F98" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G98" s="6" t="n">
@@ -8868,9 +8870,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F105" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F105" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G105" s="6" t="n">
@@ -9224,9 +9226,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F112" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F112" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G112" s="6" t="n">
@@ -9580,9 +9582,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F119" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F119" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G119" s="6" t="n">
@@ -9936,9 +9938,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F126" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F126" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G126" s="6" t="n">
@@ -12376,9 +12378,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F173" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F173" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G173" s="6" t="n">
@@ -12734,9 +12736,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F180" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F180" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G180" s="6" t="n">
@@ -13092,9 +13094,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F187" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F187" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G187" s="6" t="n">
@@ -13450,9 +13452,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F194" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F194" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G194" s="6" t="n">
@@ -13808,9 +13810,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F201" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F201" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G201" s="6" t="n">
@@ -14166,9 +14168,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F208" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F208" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G208" s="6" t="n">
@@ -14524,9 +14526,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F215" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F215" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G215" s="6" t="n">
@@ -14882,9 +14884,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F222" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F222" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G222" s="6" t="n">
@@ -17324,9 +17326,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F269" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F269" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G269" s="6" t="n">
@@ -17682,9 +17684,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F276" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F276" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G276" s="6" t="n">
@@ -18040,9 +18042,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F283" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F283" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G283" s="6" t="n">
@@ -18398,9 +18400,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F290" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F290" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G290" s="6" t="n">
@@ -18756,9 +18758,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F297" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F297" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G297" s="6" t="n">
@@ -19114,9 +19116,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F304" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F304" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G304" s="6" t="n">
@@ -19472,9 +19474,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F311" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F311" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G311" s="6" t="n">
@@ -19830,9 +19832,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F318" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F318" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G318" s="6" t="n">
@@ -22272,9 +22274,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F365" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F365" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G365" s="6" t="n">
@@ -22630,9 +22632,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F372" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F372" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G372" s="6" t="n">
@@ -22988,9 +22990,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F379" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F379" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G379" s="6" t="n">
@@ -23346,9 +23348,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F386" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F386" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G386" s="6" t="n">
@@ -23704,9 +23706,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F393" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F393" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G393" s="6" t="n">
@@ -24062,9 +24064,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F400" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F400" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G400" s="6" t="n">
@@ -24420,9 +24422,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F407" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F407" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G407" s="6" t="n">
@@ -24778,9 +24780,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F414" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F414" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G414" s="6" t="n">
@@ -27232,9 +27234,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F461" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F461" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G461" s="6" t="n">
@@ -27592,9 +27594,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F468" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F468" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G468" s="6" t="n">
@@ -27952,9 +27954,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F475" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F475" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G475" s="6" t="n">
@@ -28312,9 +28314,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F482" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F482" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G482" s="6" t="n">
@@ -28672,9 +28674,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F489" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F489" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G489" s="6" t="n">
@@ -29032,9 +29034,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F496" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F496" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G496" s="6" t="n">
@@ -29392,9 +29394,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F503" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F503" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G503" s="6" t="n">
@@ -29752,9 +29754,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F510" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F510" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G510" s="6" t="n">
@@ -32208,9 +32210,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F557" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F557" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G557" s="6" t="n">
@@ -32568,9 +32570,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F564" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F564" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G564" s="6" t="n">
@@ -32928,9 +32930,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F571" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F571" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G571" s="6" t="n">
@@ -33288,9 +33290,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F578" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F578" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G578" s="6" t="n">
@@ -33648,9 +33650,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F585" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F585" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G585" s="6" t="n">
@@ -34008,9 +34010,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F592" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F592" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G592" s="6" t="n">
@@ -34368,9 +34370,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F599" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F599" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G599" s="6" t="n">
@@ -34728,9 +34730,9 @@
           <t>L 12, L 10</t>
         </is>
       </c>
-      <c r="F606" s="29" t="inlineStr">
-        <is>
-          <t>SuTable</t>
+      <c r="F606" s="32" t="inlineStr">
+        <is>
+          <t>SigmaTau</t>
         </is>
       </c>
       <c r="G606" s="6" t="n">
@@ -35126,17 +35128,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:08</t>
+          <t>2026-10-19 21:11:37</t>
         </is>
       </c>
       <c r="D2" t="b">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9313674276604081</v>
+        <v>0.7070630607756224</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9183226402690196</v>
+        <v>0.7862695052280548</v>
       </c>
     </row>
     <row r="3">
@@ -35152,17 +35154,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:17</t>
+          <t>2026-10-19 21:11:54</t>
         </is>
       </c>
       <c r="D3" t="b">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9254286909145556</v>
+        <v>0.6793911878982013</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9081873079995147</v>
+        <v>0.7340354365328755</v>
       </c>
     </row>
     <row r="4">
@@ -35178,17 +35180,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:23</t>
+          <t>2026-10-19 21:12:04</t>
         </is>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9357644555891874</v>
+        <v>0.7124837704302815</v>
       </c>
       <c r="F4" t="n">
-        <v>0.924240939408446</v>
+        <v>0.7917517515992387</v>
       </c>
     </row>
     <row r="5">
@@ -35204,17 +35206,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:33</t>
+          <t>2026-10-19 21:12:21</t>
         </is>
       </c>
       <c r="D5" t="b">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9297990720683053</v>
+        <v>0.681465959566057</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9147546818415812</v>
+        <v>0.7388338720076649</v>
       </c>
     </row>
     <row r="6">
@@ -35230,17 +35232,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:40</t>
+          <t>2026-10-19 21:12:31</t>
         </is>
       </c>
       <c r="D6" t="b">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8978679483764915</v>
+        <v>0.6689143628316666</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8773386916253549</v>
+        <v>0.7482895397764732</v>
       </c>
     </row>
     <row r="7">
@@ -35256,17 +35258,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:49</t>
+          <t>2026-10-19 21:12:44</t>
         </is>
       </c>
       <c r="D7" t="b">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8910306774284767</v>
+        <v>0.6477192091893146</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8628324254543914</v>
+        <v>0.7006326438593266</v>
       </c>
     </row>
     <row r="8">
@@ -35282,17 +35284,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-30 11:00:55</t>
+          <t>2026-10-19 21:12:55</t>
         </is>
       </c>
       <c r="D8" t="b">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1.156031848570945</v>
+        <v>0.6840308372154181</v>
       </c>
       <c r="F8" t="n">
-        <v>1.110277740774374</v>
+        <v>0.7651162276518461</v>
       </c>
     </row>
     <row r="9">
@@ -35308,17 +35310,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:03</t>
+          <t>2026-10-19 21:13:08</t>
         </is>
       </c>
       <c r="D9" t="b">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>1.045982500461952</v>
+        <v>0.6611728787787279</v>
       </c>
       <c r="F9" t="n">
-        <v>1.110277740774374</v>
+        <v>0.7158320916385558</v>
       </c>
     </row>
     <row r="10">
@@ -35334,17 +35336,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:09</t>
+          <t>2026-10-19 21:13:19</t>
         </is>
       </c>
       <c r="D10" t="b">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>1.195672752269585</v>
+        <v>0.7020568837415596</v>
       </c>
       <c r="F10" t="n">
-        <v>1.143001667251261</v>
+        <v>0.7806625217388528</v>
       </c>
     </row>
     <row r="11">
@@ -35360,17 +35362,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:19</t>
+          <t>2026-10-19 21:13:36</t>
         </is>
       </c>
       <c r="D11" t="b">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1.071221376346925</v>
+        <v>0.6743828231536745</v>
       </c>
       <c r="F11" t="n">
-        <v>1.143001667251261</v>
+        <v>0.7295058797486463</v>
       </c>
     </row>
     <row r="12">
@@ -35386,17 +35388,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:24</t>
+          <t>2026-10-19 21:13:47</t>
         </is>
       </c>
       <c r="D12" t="b">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1.412353769049239</v>
+        <v>0.7514164230972632</v>
       </c>
       <c r="F12" t="n">
-        <v>1.342101653506674</v>
+        <v>0.8786530958528124</v>
       </c>
     </row>
     <row r="13">
@@ -35412,17 +35414,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:32</t>
+          <t>2026-10-19 21:14:03</t>
         </is>
       </c>
       <c r="D13" t="b">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>1.287010165537356</v>
+        <v>0.7381296990282354</v>
       </c>
       <c r="F13" t="n">
-        <v>1.333336873905144</v>
+        <v>0.8119512812152355</v>
       </c>
     </row>
     <row r="14">
@@ -35438,17 +35440,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:40</t>
+          <t>2026-10-19 21:14:13</t>
         </is>
       </c>
       <c r="D14" t="b">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>1.462138387556376</v>
+        <v>0.7654739981355015</v>
       </c>
       <c r="F14" t="n">
-        <v>1.388685579638923</v>
+        <v>0.8985790621405119</v>
       </c>
     </row>
     <row r="15">
@@ -35464,17 +35466,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:49</t>
+          <t>2026-10-19 21:14:26</t>
         </is>
       </c>
       <c r="D15" t="b">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>1.314551760971658</v>
+        <v>0.7623140170229591</v>
       </c>
       <c r="F15" t="n">
-        <v>1.363828323487535</v>
+        <v>0.8267906573731005</v>
       </c>
     </row>
     <row r="16">
@@ -35490,17 +35492,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-06-30 11:01:56</t>
+          <t>2026-10-19 21:14:36</t>
         </is>
       </c>
       <c r="D16" t="b">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6447473434995034</v>
+        <v>0.836156837502493</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7294068029095861</v>
+        <v>0.9267664007388728</v>
       </c>
     </row>
     <row r="17">
@@ -35516,17 +35518,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:06</t>
+          <t>2026-10-19 21:14:52</t>
         </is>
       </c>
       <c r="D17" t="b">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0.6874992517490198</v>
+        <v>0.826707269006937</v>
       </c>
       <c r="F17" t="n">
-        <v>0.700470179149252</v>
+        <v>0.8956723384319335</v>
       </c>
     </row>
     <row r="18">
@@ -35542,17 +35544,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:12</t>
+          <t>2026-10-19 21:15:03</t>
         </is>
       </c>
       <c r="D18" t="b">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6594533356492267</v>
+        <v>0.865068758112547</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7455307007834006</v>
+        <v>0.9568151499677057</v>
       </c>
     </row>
     <row r="19">
@@ -35568,17 +35570,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:21</t>
+          <t>2026-10-19 21:15:16</t>
         </is>
       </c>
       <c r="D19" t="b">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6518177506528604</v>
+        <v>0.8516740645479524</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7190479702131533</v>
+        <v>0.9206773501423333</v>
       </c>
     </row>
     <row r="20">
@@ -35594,17 +35596,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:30</t>
+          <t>2026-10-19 21:15:29</t>
         </is>
       </c>
       <c r="D20" t="b">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6480582035145244</v>
+        <v>0.8429615633564104</v>
       </c>
       <c r="F20" t="n">
-        <v>0.7362154980937871</v>
+        <v>0.933224178953452</v>
       </c>
     </row>
     <row r="21">
@@ -35620,17 +35622,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:44</t>
+          <t>2026-10-19 21:15:46</t>
         </is>
       </c>
       <c r="D21" t="b">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6919995148513416</v>
+        <v>0.8314455727992435</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7060725371020858</v>
+        <v>0.9011196221176471</v>
       </c>
     </row>
     <row r="22">
@@ -35646,17 +35648,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-06-30 11:02:53</t>
+          <t>2026-10-19 21:15:56</t>
         </is>
       </c>
       <c r="D22" t="b">
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>0.663092822627384</v>
+        <v>0.8713654647956686</v>
       </c>
       <c r="F22" t="n">
-        <v>0.752406821079271</v>
+        <v>0.9633815514162125</v>
       </c>
     </row>
     <row r="23">
@@ -35672,17 +35674,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:08</t>
+          <t>2026-10-19 21:16:09</t>
         </is>
       </c>
       <c r="D23" t="b">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0.6553272828276429</v>
+        <v>0.8568541126548624</v>
       </c>
       <c r="F23" t="n">
-        <v>0.7248387627473158</v>
+        <v>0.9262165546179364</v>
       </c>
     </row>
     <row r="24">
@@ -35698,17 +35700,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:14</t>
+          <t>2026-10-19 21:16:22</t>
         </is>
       </c>
       <c r="D24" t="b">
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6246851185848359</v>
+        <v>0.7986034627384012</v>
       </c>
       <c r="F24" t="n">
-        <v>0.6827549715591454</v>
+        <v>0.882173950352976</v>
       </c>
     </row>
     <row r="25">
@@ -35724,17 +35726,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:23</t>
+          <t>2026-10-19 21:16:38</t>
         </is>
       </c>
       <c r="D25" t="b">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6130733788317149</v>
+        <v>0.7938857397531466</v>
       </c>
       <c r="F25" t="n">
-        <v>0.6613645241687596</v>
+        <v>0.8577728635606202</v>
       </c>
     </row>
     <row r="26">
@@ -35750,17 +35752,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:30</t>
+          <t>2026-10-19 21:16:49</t>
         </is>
       </c>
       <c r="D26" t="b">
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6338984094320581</v>
+        <v>0.8215908265449891</v>
       </c>
       <c r="F26" t="n">
-        <v>0.6984083643629335</v>
+        <v>0.9114741164483243</v>
       </c>
     </row>
     <row r="27">
@@ -35776,17 +35778,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:39</t>
+          <t>2026-10-19 21:17:01</t>
         </is>
       </c>
       <c r="D27" t="b">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>0.6268492725713898</v>
+        <v>0.8153208225603749</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6790902364428459</v>
+        <v>0.8821436767956965</v>
       </c>
     </row>
     <row r="28">
@@ -35802,17 +35804,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:45</t>
+          <t>2026-10-19 21:17:11</t>
         </is>
       </c>
       <c r="D28" t="b">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7040692320842973</v>
+        <v>0.7069279325266725</v>
       </c>
       <c r="F28" t="n">
-        <v>0.7022841612597917</v>
+        <v>0.8117302419793929</v>
       </c>
     </row>
     <row r="29">
@@ -35828,17 +35830,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:52</t>
+          <t>2026-10-19 21:17:24</t>
         </is>
       </c>
       <c r="D29" t="b">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>0.6721800049537465</v>
+        <v>0.655330037176063</v>
       </c>
       <c r="F29" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="30">
@@ -35854,17 +35856,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-06-30 11:03:58</t>
+          <t>2026-10-19 21:17:34</t>
         </is>
       </c>
       <c r="D30" t="b">
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7126660139940455</v>
+        <v>0.7186359334148086</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7099618107091675</v>
+        <v>0.799565295467869</v>
       </c>
     </row>
     <row r="31">
@@ -35880,17 +35882,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:06</t>
+          <t>2026-10-19 21:17:47</t>
         </is>
       </c>
       <c r="D31" t="b">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0.6601593344457493</v>
+        <v>0.6476692725933388</v>
       </c>
       <c r="F31" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="32">
@@ -35906,17 +35908,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:11</t>
+          <t>2026-10-19 21:17:57</t>
         </is>
       </c>
       <c r="D32" t="b">
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>0.7080025395719465</v>
+        <v>0.7125704268453913</v>
       </c>
       <c r="F32" t="n">
-        <v>0.7076258936695208</v>
+        <v>0.8203941209914902</v>
       </c>
     </row>
     <row r="33">
@@ -35932,17 +35934,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:19</t>
+          <t>2026-10-19 21:18:09</t>
         </is>
       </c>
       <c r="D33" t="b">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>0.6762660222489462</v>
+        <v>0.6590459086039478</v>
       </c>
       <c r="F33" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="34">
@@ -35958,17 +35960,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:24</t>
+          <t>2026-10-19 21:18:19</t>
         </is>
       </c>
       <c r="D34" t="b">
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>0.7166346468420913</v>
+        <v>0.7242690345009702</v>
       </c>
       <c r="F34" t="n">
-        <v>0.7153372868452239</v>
+        <v>0.808182799912326</v>
       </c>
     </row>
     <row r="35">
@@ -35984,17 +35986,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:32</t>
+          <t>2026-10-19 21:18:33</t>
         </is>
       </c>
       <c r="D35" t="b">
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>0.6652671800925478</v>
+        <v>0.6526224871224137</v>
       </c>
       <c r="F35" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="36">
@@ -36010,17 +36012,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:37</t>
+          <t>2026-10-19 21:18:43</t>
         </is>
       </c>
       <c r="D36" t="b">
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>0.6766917202969444</v>
+        <v>0.668163716077495</v>
       </c>
       <c r="F36" t="n">
-        <v>0.6476971618162031</v>
+        <v>0.7527257002049141</v>
       </c>
     </row>
     <row r="37">
@@ -36036,17 +36038,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:45</t>
+          <t>2026-10-19 21:18:55</t>
         </is>
       </c>
       <c r="D37" t="b">
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>0.644363413581808</v>
+        <v>0.6159832728781551</v>
       </c>
       <c r="F37" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="38">
@@ -36062,17 +36064,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:51</t>
+          <t>2026-10-19 21:19:05</t>
         </is>
       </c>
       <c r="D38" t="b">
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>0.6850578252280251</v>
+        <v>0.6674769316850493</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6491002486137135</v>
+        <v>0.7408868627213845</v>
       </c>
     </row>
     <row r="39">
@@ -36088,17 +36090,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-06-30 11:04:59</t>
+          <t>2026-10-19 21:19:18</t>
         </is>
       </c>
       <c r="D39" t="b">
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>0.6277279350167287</v>
+        <v>0.6060421988665661</v>
       </c>
       <c r="F39" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="40">
@@ -36114,17 +36116,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:05</t>
+          <t>2026-10-19 21:19:28</t>
         </is>
       </c>
       <c r="D40" t="b">
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>0.9715996269709197</v>
+        <v>0.6859977668578917</v>
       </c>
       <c r="F40" t="n">
-        <v>0.9463063133842711</v>
+        <v>0.7798935440204997</v>
       </c>
     </row>
     <row r="41">
@@ -36140,17 +36142,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:13</t>
+          <t>2026-10-19 21:19:42</t>
         </is>
       </c>
       <c r="D41" t="b">
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>0.9550977139315759</v>
+        <v>0.6388058104868259</v>
       </c>
       <c r="F41" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="42">
@@ -36166,17 +36168,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:19</t>
+          <t>2026-10-19 21:19:53</t>
         </is>
       </c>
       <c r="D42" t="b">
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>0.9779997926075252</v>
+        <v>0.6886720332088317</v>
       </c>
       <c r="F42" t="n">
-        <v>0.9501714158621705</v>
+        <v>0.7678992615557168</v>
       </c>
     </row>
     <row r="43">
@@ -36192,17 +36194,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:28</t>
+          <t>2026-10-19 21:20:07</t>
         </is>
       </c>
       <c r="D43" t="b">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>0.9602228849900853</v>
+        <v>0.6244129389026396</v>
       </c>
       <c r="F43" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="44">
@@ -36218,17 +36220,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:34</t>
+          <t>2026-10-19 21:20:18</t>
         </is>
       </c>
       <c r="D44" t="b">
         <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>1.007245628347618</v>
+        <v>0.701910658727848</v>
       </c>
       <c r="F44" t="n">
-        <v>0.9859600797022288</v>
+        <v>0.8041031028462403</v>
       </c>
     </row>
     <row r="45">
@@ -36244,17 +36246,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:43</t>
+          <t>2026-10-19 21:20:31</t>
         </is>
       </c>
       <c r="D45" t="b">
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>0.9911973288468772</v>
+        <v>0.6512604410815346</v>
       </c>
       <c r="F45" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="46">
@@ -36270,17 +36272,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-06-30 11:05:51</t>
+          <t>2026-10-19 21:20:42</t>
         </is>
       </c>
       <c r="D46" t="b">
         <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>1.013645847319352</v>
+        <v>0.7136183147267252</v>
       </c>
       <c r="F46" t="n">
-        <v>0.9898252237348545</v>
+        <v>0.7919775601778436</v>
       </c>
     </row>
     <row r="47">
@@ -36296,17 +36298,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:08</t>
+          <t>2026-10-19 21:20:56</t>
         </is>
       </c>
       <c r="D47" t="b">
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>0.9757510259496611</v>
+        <v>0.6428926919008761</v>
       </c>
       <c r="F47" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="48">
@@ -36322,17 +36324,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:15</t>
+          <t>2026-10-19 21:21:06</t>
         </is>
       </c>
       <c r="D48" t="b">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>1.241851271974181</v>
+        <v>0.8041562148298101</v>
       </c>
       <c r="F48" t="n">
-        <v>1.224218905820375</v>
+        <v>0.9235567105875038</v>
       </c>
     </row>
     <row r="49">
@@ -36348,17 +36350,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:24</t>
+          <t>2026-10-19 21:21:21</t>
         </is>
       </c>
       <c r="D49" t="b">
         <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>1.136114277323288</v>
+        <v>0.7271257791735245</v>
       </c>
       <c r="F49" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="50">
@@ -36374,17 +36376,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:30</t>
+          <t>2026-10-19 21:21:31</t>
         </is>
       </c>
       <c r="D50" t="b">
         <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>1.24841538600271</v>
+        <v>0.8157131938574915</v>
       </c>
       <c r="F50" t="n">
-        <v>1.228084219489427</v>
+        <v>0.9368059401319186</v>
       </c>
     </row>
     <row r="51">
@@ -36400,17 +36402,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:39</t>
+          <t>2026-10-19 21:21:44</t>
         </is>
       </c>
       <c r="D51" t="b">
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>1.14189472459448</v>
+        <v>0.7299379150900345</v>
       </c>
       <c r="F51" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="52">
@@ -36426,17 +36428,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-06-30 11:06:45</t>
+          <t>2026-10-19 21:21:55</t>
         </is>
       </c>
       <c r="D52" t="b">
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>1.292882344575017</v>
+        <v>0.8230475086923286</v>
       </c>
       <c r="F52" t="n">
-        <v>1.280549981953451</v>
+        <v>0.9440301828635675</v>
       </c>
     </row>
     <row r="53">
@@ -36452,17 +36454,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:01</t>
+          <t>2026-10-19 21:22:09</t>
         </is>
       </c>
       <c r="D53" t="b">
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>1.162580667089709</v>
+        <v>0.7411642336499212</v>
       </c>
       <c r="F53" t="n">
-        <v>0.2629935900392255</v>
+        <v>0.4350793802622716</v>
       </c>
     </row>
     <row r="54">
@@ -36478,17 +36480,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:07</t>
+          <t>2026-10-19 21:22:20</t>
         </is>
       </c>
       <c r="D54" t="b">
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>1.299446474164108</v>
+        <v>0.834766868856173</v>
       </c>
       <c r="F54" t="n">
-        <v>1.284415322404287</v>
+        <v>0.9574479785947339</v>
       </c>
     </row>
     <row r="55">
@@ -36504,17 +36506,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:18</t>
+          <t>2026-10-19 21:22:34</t>
         </is>
       </c>
       <c r="D55" t="b">
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>1.168333201128731</v>
+        <v>0.7466407424680058</v>
       </c>
       <c r="F55" t="n">
-        <v>0.274424270405801</v>
+        <v>0.4495314589172049</v>
       </c>
     </row>
     <row r="56">
@@ -36530,17 +36532,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:25</t>
+          <t>2026-10-19 21:22:48</t>
         </is>
       </c>
       <c r="D56" t="b">
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>0.7484425910310099</v>
+        <v>0.8756453607376016</v>
       </c>
       <c r="F56" t="n">
-        <v>0.7778731761682889</v>
+        <v>0.9724583971098698</v>
       </c>
     </row>
     <row r="57">
@@ -36556,17 +36558,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:40</t>
+          <t>2026-10-19 21:23:10</t>
         </is>
       </c>
       <c r="D57" t="b">
         <v>0</v>
       </c>
       <c r="E57" t="n">
-        <v>0.7812610601545065</v>
+        <v>0.8710034801819637</v>
       </c>
       <c r="F57" t="n">
-        <v>0.7422474564975553</v>
+        <v>0.947818642068927</v>
       </c>
     </row>
     <row r="58">
@@ -36582,17 +36584,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:46</t>
+          <t>2026-10-19 21:23:22</t>
         </is>
       </c>
       <c r="D58" t="b">
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>0.7695323724817863</v>
+        <v>0.9247909643171731</v>
       </c>
       <c r="F58" t="n">
-        <v>0.796128366142852</v>
+        <v>1.007992454010695</v>
       </c>
     </row>
     <row r="59">
@@ -36608,17 +36610,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-06-30 11:07:56</t>
+          <t>2026-10-19 21:23:44</t>
         </is>
       </c>
       <c r="D59" t="b">
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>0.8138470976043788</v>
+        <v>0.9146589375361638</v>
       </c>
       <c r="F59" t="n">
-        <v>0.7614028527268306</v>
+        <v>0.9849431937159778</v>
       </c>
     </row>
     <row r="60">
@@ -36634,17 +36636,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:04</t>
+          <t>2026-10-19 21:23:56</t>
         </is>
       </c>
       <c r="D60" t="b">
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>0.7525358107491352</v>
+        <v>0.8818803453317099</v>
       </c>
       <c r="F60" t="n">
-        <v>0.7848824621700692</v>
+        <v>0.979051532455641</v>
       </c>
     </row>
     <row r="61">
@@ -36660,17 +36662,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:14</t>
+          <t>2026-10-19 21:24:18</t>
         </is>
       </c>
       <c r="D61" t="b">
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>0.7592587164850815</v>
+        <v>0.8764812010829951</v>
       </c>
       <c r="F61" t="n">
-        <v>0.7476008166399717</v>
+        <v>0.9534559838654962</v>
       </c>
     </row>
     <row r="62">
@@ -36686,17 +36688,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:21</t>
+          <t>2026-10-19 21:24:31</t>
         </is>
       </c>
       <c r="D62" t="b">
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>0.7737133703519815</v>
+        <v>0.9303751285056207</v>
       </c>
       <c r="F62" t="n">
-        <v>0.8032115544804324</v>
+        <v>1.014946674540917</v>
       </c>
     </row>
     <row r="63">
@@ -36712,17 +36714,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:30</t>
+          <t>2026-10-19 21:24:51</t>
         </is>
       </c>
       <c r="D63" t="b">
         <v>0</v>
       </c>
       <c r="E63" t="n">
-        <v>0.8193504978043743</v>
+        <v>0.9205971787909931</v>
       </c>
       <c r="F63" t="n">
-        <v>0.7668390062325611</v>
+        <v>0.9906823705196349</v>
       </c>
     </row>
     <row r="64">
@@ -36738,17 +36740,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:35</t>
+          <t>2026-10-19 21:25:03</t>
         </is>
       </c>
       <c r="D64" t="b">
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>0.719764184314919</v>
+        <v>0.8342543261412836</v>
       </c>
       <c r="F64" t="n">
-        <v>0.7298228927479042</v>
+        <v>0.9265971047864976</v>
       </c>
     </row>
     <row r="65">
@@ -36764,17 +36766,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:44</t>
+          <t>2026-10-19 21:25:22</t>
         </is>
       </c>
       <c r="D65" t="b">
         <v>0</v>
       </c>
       <c r="E65" t="n">
-        <v>0.7813470299390506</v>
+        <v>0.8244137089308168</v>
       </c>
       <c r="F65" t="n">
-        <v>0.7037464115537873</v>
+        <v>0.9086085187360482</v>
       </c>
     </row>
     <row r="66">
@@ -36790,17 +36792,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:50</t>
+          <t>2026-10-19 21:25:34</t>
         </is>
       </c>
       <c r="D66" t="b">
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>0.7402518491872198</v>
+        <v>0.8708093045666444</v>
       </c>
       <c r="F66" t="n">
-        <v>0.7475638244538184</v>
+        <v>0.949172176134264</v>
       </c>
     </row>
     <row r="67">
@@ -36816,17 +36818,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-06-30 11:08:58</t>
+          <t>2026-10-19 21:25:51</t>
         </is>
       </c>
       <c r="D67" t="b">
         <v>0</v>
       </c>
       <c r="E67" t="n">
-        <v>0.8313369513694192</v>
+        <v>0.8741776211450201</v>
       </c>
       <c r="F67" t="n">
-        <v>0.7224904062429726</v>
+        <v>0.9421901388902688</v>
       </c>
     </row>
     <row r="68">
@@ -36842,17 +36844,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:04</t>
+          <t>2026-10-19 21:26:03</t>
         </is>
       </c>
       <c r="D68" t="b">
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>1.013272284862945</v>
+        <v>0.8540758168973267</v>
       </c>
       <c r="F68" t="n">
-        <v>1.019320033325171</v>
+        <v>0.9466649078462732</v>
       </c>
     </row>
     <row r="69">
@@ -36868,17 +36870,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:12</t>
+          <t>2026-10-19 21:26:20</t>
         </is>
       </c>
       <c r="D69" t="b">
         <v>0</v>
       </c>
       <c r="E69" t="n">
-        <v>0.9350941891681576</v>
+        <v>0.8428875910035569</v>
       </c>
       <c r="F69" t="n">
-        <v>1.019320033325171</v>
+        <v>0.9259569854473427</v>
       </c>
     </row>
     <row r="70">
@@ -36894,17 +36896,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:18</t>
+          <t>2026-10-19 21:26:32</t>
         </is>
       </c>
       <c r="D70" t="b">
         <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>1.030320989548137</v>
+        <v>0.8913277810942775</v>
       </c>
       <c r="F70" t="n">
-        <v>1.037534388928505</v>
+        <v>0.9764760431500022</v>
       </c>
     </row>
     <row r="71">
@@ -36920,17 +36922,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:27</t>
+          <t>2026-10-19 21:26:52</t>
         </is>
       </c>
       <c r="D71" t="b">
         <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>0.9615934594913033</v>
+        <v>0.8939010948885404</v>
       </c>
       <c r="F71" t="n">
-        <v>1.037534388928505</v>
+        <v>0.9625745905646153</v>
       </c>
     </row>
     <row r="72">
@@ -36946,17 +36948,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:33</t>
+          <t>2026-10-19 21:27:04</t>
         </is>
       </c>
       <c r="D72" t="b">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>1.048932009665137</v>
+        <v>0.869787584567179</v>
       </c>
       <c r="F72" t="n">
-        <v>1.058974506660843</v>
+        <v>0.9655765980555255</v>
       </c>
     </row>
     <row r="73">
@@ -36972,17 +36974,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:44</t>
+          <t>2026-10-19 21:27:23</t>
         </is>
       </c>
       <c r="D73" t="b">
         <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>0.9637381558105287</v>
+        <v>0.8662069949477491</v>
       </c>
       <c r="F73" t="n">
-        <v>1.057929931965285</v>
+        <v>0.9420003217184159</v>
       </c>
     </row>
     <row r="74">
@@ -36998,17 +37000,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-06-30 11:09:53</t>
+          <t>2026-10-19 21:27:35</t>
         </is>
       </c>
       <c r="D74" t="b">
         <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>1.065170547872711</v>
+        <v>0.9187489661571159</v>
       </c>
       <c r="F74" t="n">
-        <v>1.071929276470895</v>
+        <v>1.000407325879195</v>
       </c>
     </row>
     <row r="75">
@@ -37024,17 +37026,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:04</t>
+          <t>2026-10-19 21:27:54</t>
         </is>
       </c>
       <c r="D75" t="b">
         <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>0.9904436723854734</v>
+        <v>0.9100262542182401</v>
       </c>
       <c r="F75" t="n">
-        <v>1.062678904992403</v>
+        <v>0.9789397928199073</v>
       </c>
     </row>
     <row r="76">
@@ -37050,17 +37052,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:11</t>
+          <t>2026-10-19 21:28:06</t>
         </is>
       </c>
       <c r="D76" t="b">
         <v>1</v>
       </c>
       <c r="E76" t="n">
-        <v>1.270526214848734</v>
+        <v>0.9901187389820735</v>
       </c>
       <c r="F76" t="n">
-        <v>1.270171216779049</v>
+        <v>1.084446669397788</v>
       </c>
     </row>
     <row r="77">
@@ -37076,17 +37078,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:19</t>
+          <t>2026-10-19 21:28:23</t>
         </is>
       </c>
       <c r="D77" t="b">
         <v>0</v>
       </c>
       <c r="E77" t="n">
-        <v>1.147804574311298</v>
+        <v>0.9484686022919958</v>
       </c>
       <c r="F77" t="n">
-        <v>1.173189009696141</v>
+        <v>1.042108311615036</v>
       </c>
     </row>
     <row r="78">
@@ -37102,17 +37104,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:25</t>
+          <t>2026-10-19 21:28:35</t>
         </is>
       </c>
       <c r="D78" t="b">
         <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>1.283158993217288</v>
+        <v>1.034724915237148</v>
       </c>
       <c r="F78" t="n">
-        <v>1.274721176337783</v>
+        <v>1.12226949089135</v>
       </c>
     </row>
     <row r="79">
@@ -37128,17 +37130,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:33</t>
+          <t>2026-10-19 21:28:51</t>
         </is>
       </c>
       <c r="D79" t="b">
         <v>0</v>
       </c>
       <c r="E79" t="n">
-        <v>1.162938397166476</v>
+        <v>0.997550238455824</v>
       </c>
       <c r="F79" t="n">
-        <v>1.214271685043685</v>
+        <v>1.081011294103167</v>
       </c>
     </row>
     <row r="80">
@@ -37154,17 +37156,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:39</t>
+          <t>2026-10-19 21:29:03</t>
         </is>
       </c>
       <c r="D80" t="b">
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>1.321266670947431</v>
+        <v>1.012497087982881</v>
       </c>
       <c r="F80" t="n">
-        <v>1.317411384558224</v>
+        <v>1.109194680535227</v>
       </c>
     </row>
     <row r="81">
@@ -37180,17 +37182,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:47</t>
+          <t>2026-10-19 21:29:19</t>
         </is>
       </c>
       <c r="D81" t="b">
         <v>0</v>
       </c>
       <c r="E81" t="n">
-        <v>1.188891148639416</v>
+        <v>0.9655524192582856</v>
       </c>
       <c r="F81" t="n">
-        <v>1.173189009696141</v>
+        <v>1.062315809786592</v>
       </c>
     </row>
     <row r="82">
@@ -37206,17 +37208,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-06-30 11:10:55</t>
+          <t>2026-10-19 21:29:31</t>
         </is>
       </c>
       <c r="D82" t="b">
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>1.333731219604333</v>
+        <v>1.058077167998294</v>
       </c>
       <c r="F82" t="n">
-        <v>1.321963420472743</v>
+        <v>1.147282099881837</v>
       </c>
     </row>
     <row r="83">
@@ -37232,17 +37234,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:04</t>
+          <t>2026-10-19 21:29:47</t>
         </is>
       </c>
       <c r="D83" t="b">
         <v>0</v>
       </c>
       <c r="E83" t="n">
-        <v>1.204072854568345</v>
+        <v>1.014708492984322</v>
       </c>
       <c r="F83" t="n">
-        <v>1.214271685043685</v>
+        <v>1.101895159473141</v>
       </c>
     </row>
     <row r="84">
@@ -37258,17 +37260,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:13</t>
+          <t>2026-10-19 21:30:00</t>
         </is>
       </c>
       <c r="D84" t="b">
         <v>1</v>
       </c>
       <c r="E84" t="n">
-        <v>0.739748208041207</v>
+        <v>0.8598213081400777</v>
       </c>
       <c r="F84" t="n">
-        <v>0.7672321216330761</v>
+        <v>0.9523072543082783</v>
       </c>
     </row>
     <row r="85">
@@ -37284,17 +37286,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:26</t>
+          <t>2026-10-19 21:30:16</t>
         </is>
       </c>
       <c r="D85" t="b">
         <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>0.764144031011288</v>
+        <v>0.8394783213516731</v>
       </c>
       <c r="F85" t="n">
-        <v>0.7291949521109035</v>
+        <v>0.9222380822106006</v>
       </c>
     </row>
     <row r="86">
@@ -37310,17 +37312,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:31</t>
+          <t>2026-10-19 21:30:28</t>
         </is>
       </c>
       <c r="D86" t="b">
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>0.7581121699476271</v>
+        <v>0.891765406331301</v>
       </c>
       <c r="F86" t="n">
-        <v>0.7838266376249012</v>
+        <v>0.9858146218637234</v>
       </c>
     </row>
     <row r="87">
@@ -37336,17 +37338,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:39</t>
+          <t>2026-10-19 21:30:44</t>
         </is>
       </c>
       <c r="D87" t="b">
         <v>0</v>
       </c>
       <c r="E87" t="n">
-        <v>0.7953429026013189</v>
+        <v>0.8762740992165986</v>
       </c>
       <c r="F87" t="n">
-        <v>0.7461781049713321</v>
+        <v>0.9570028535061436</v>
       </c>
     </row>
     <row r="88">
@@ -37362,17 +37364,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-06-30 11:11:48</t>
+          <t>2026-10-19 21:30:56</t>
         </is>
       </c>
       <c r="D88" t="b">
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>0.743808911448973</v>
+        <v>0.8660555884092178</v>
       </c>
       <c r="F88" t="n">
-        <v>0.7741979065568481</v>
+        <v>0.9588575112062865</v>
       </c>
     </row>
     <row r="89">
@@ -37388,17 +37390,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:01</t>
+          <t>2026-10-19 21:31:11</t>
         </is>
       </c>
       <c r="D89" t="b">
         <v>0</v>
       </c>
       <c r="E89" t="n">
-        <v>0.7606010528999037</v>
+        <v>0.8446332215165508</v>
       </c>
       <c r="F89" t="n">
-        <v>0.7344912707368871</v>
+        <v>0.9277829760735681</v>
       </c>
     </row>
     <row r="90">
@@ -37414,17 +37416,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:07</t>
+          <t>2026-10-19 21:31:24</t>
         </is>
       </c>
       <c r="D90" t="b">
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>0.7622486932516287</v>
+        <v>0.8977973862750824</v>
       </c>
       <c r="F90" t="n">
-        <v>0.790860126218396</v>
+        <v>0.9924524689915516</v>
       </c>
     </row>
     <row r="91">
@@ -37440,17 +37442,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:20</t>
+          <t>2026-10-19 21:31:39</t>
         </is>
       </c>
       <c r="D91" t="b">
         <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>0.7996509228646478</v>
+        <v>0.8820469676654232</v>
       </c>
       <c r="F91" t="n">
-        <v>0.7515485434123217</v>
+        <v>0.9626730193008901</v>
       </c>
     </row>
     <row r="92">
@@ -37466,17 +37468,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:29</t>
+          <t>2026-10-19 21:31:52</t>
         </is>
       </c>
       <c r="D92" t="b">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>0.7112986599604337</v>
+        <v>0.8168526695825841</v>
       </c>
       <c r="F92" t="n">
-        <v>0.7194847828923929</v>
+        <v>0.9070774250333219</v>
       </c>
     </row>
     <row r="93">
@@ -37492,17 +37494,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:37</t>
+          <t>2026-10-19 21:32:08</t>
         </is>
       </c>
       <c r="D93" t="b">
         <v>0</v>
       </c>
       <c r="E93" t="n">
-        <v>0.7613268001290862</v>
+        <v>0.8023521117636634</v>
       </c>
       <c r="F93" t="n">
-        <v>0.6921420387508209</v>
+        <v>0.8836651746805491</v>
       </c>
     </row>
     <row r="94">
@@ -37518,17 +37520,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:44</t>
+          <t>2026-10-19 21:32:20</t>
         </is>
       </c>
       <c r="D94" t="b">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>0.7293092035909696</v>
+        <v>0.8468515825830343</v>
       </c>
       <c r="F94" t="n">
-        <v>0.7356078822297355</v>
+        <v>0.9338039616578574</v>
       </c>
     </row>
     <row r="95">
@@ -37544,17 +37546,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:52</t>
+          <t>2026-10-19 21:32:35</t>
         </is>
       </c>
       <c r="D95" t="b">
         <v>0</v>
       </c>
       <c r="E95" t="n">
-        <v>0.819594511490375</v>
+        <v>0.8354974099855401</v>
       </c>
       <c r="F95" t="n">
-        <v>0.7089482962782931</v>
+        <v>0.9175666220854458</v>
       </c>
     </row>
     <row r="96">
@@ -37570,17 +37572,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2026-06-30 11:12:59</t>
+          <t>2026-10-19 21:32:46</t>
         </is>
       </c>
       <c r="D96" t="b">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>1.005921542045707</v>
+        <v>0.8331967654172886</v>
       </c>
       <c r="F96" t="n">
-        <v>1.00906477697205</v>
+        <v>0.9269832029865707</v>
       </c>
     </row>
     <row r="97">
@@ -37596,17 +37598,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:08</t>
+          <t>2026-10-19 21:33:01</t>
         </is>
       </c>
       <c r="D97" t="b">
         <v>0</v>
       </c>
       <c r="E97" t="n">
-        <v>0.9278850868149607</v>
+        <v>0.8254928159653835</v>
       </c>
       <c r="F97" t="n">
-        <v>1.00906477697205</v>
+        <v>0.9007828210680328</v>
       </c>
     </row>
     <row r="98">
@@ -37622,17 +37624,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:14</t>
+          <t>2026-10-19 21:33:13</t>
         </is>
       </c>
       <c r="D98" t="b">
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>1.021724601202592</v>
+        <v>0.8692113108793487</v>
       </c>
       <c r="F98" t="n">
-        <v>1.025692282135532</v>
+        <v>0.9600253844280481</v>
       </c>
     </row>
     <row r="99">
@@ -37648,17 +37650,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:23</t>
+          <t>2026-10-19 21:33:27</t>
         </is>
       </c>
       <c r="D99" t="b">
         <v>0</v>
       </c>
       <c r="E99" t="n">
-        <v>0.9524738156671918</v>
+        <v>0.8547431395032338</v>
       </c>
       <c r="F99" t="n">
-        <v>1.025692282135532</v>
+        <v>0.9349963427215459</v>
       </c>
     </row>
     <row r="100">
@@ -37674,17 +37676,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:29</t>
+          <t>2026-10-19 21:33:40</t>
         </is>
       </c>
       <c r="D100" t="b">
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>1.041253844721456</v>
+        <v>0.8542208295027043</v>
       </c>
       <c r="F100" t="n">
-        <v>1.048719160176225</v>
+        <v>0.9455304639301365</v>
       </c>
     </row>
     <row r="101">
@@ -37700,17 +37702,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:37</t>
+          <t>2026-10-19 21:33:59</t>
         </is>
       </c>
       <c r="D101" t="b">
         <v>0</v>
       </c>
       <c r="E101" t="n">
-        <v>0.9678606869401135</v>
+        <v>0.834859866487164</v>
       </c>
       <c r="F101" t="n">
-        <v>1.047668890999291</v>
+        <v>0.9165679218479522</v>
       </c>
     </row>
     <row r="102">
@@ -37726,17 +37728,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:43</t>
+          <t>2026-10-19 21:34:11</t>
         </is>
       </c>
       <c r="D102" t="b">
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>1.056574126888789</v>
+        <v>0.8859131877885023</v>
       </c>
       <c r="F102" t="n">
-        <v>1.065346810119878</v>
+        <v>0.9788511379429043</v>
       </c>
     </row>
     <row r="103">
@@ -37752,17 +37754,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:51</t>
+          <t>2026-10-19 21:34:26</t>
         </is>
       </c>
       <c r="D103" t="b">
         <v>0</v>
       </c>
       <c r="E103" t="n">
-        <v>0.9813239964703264</v>
+        <v>0.8714338350698277</v>
       </c>
       <c r="F103" t="n">
-        <v>1.051903964868142</v>
+        <v>0.9511320195855147</v>
       </c>
     </row>
     <row r="104">
@@ -37778,17 +37780,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2026-06-30 11:13:56</t>
+          <t>2026-10-19 21:34:37</t>
         </is>
       </c>
       <c r="D104" t="b">
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>1.268674390646135</v>
+        <v>0.966188735470932</v>
       </c>
       <c r="F104" t="n">
-        <v>1.265653427671221</v>
+        <v>1.063503797586827</v>
       </c>
     </row>
     <row r="105">
@@ -37804,17 +37806,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:06</t>
+          <t>2026-10-19 21:34:51</t>
         </is>
       </c>
       <c r="D105" t="b">
         <v>0</v>
       </c>
       <c r="E105" t="n">
-        <v>1.139702241408047</v>
+        <v>0.9211314084245805</v>
       </c>
       <c r="F105" t="n">
-        <v>1.050747242268714</v>
+        <v>1.01505457800391</v>
       </c>
     </row>
     <row r="106">
@@ -37830,17 +37832,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:12</t>
+          <t>2026-10-19 21:35:03</t>
         </is>
       </c>
       <c r="D106" t="b">
         <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>1.274678751781434</v>
+        <v>1.00750396033467</v>
       </c>
       <c r="F106" t="n">
-        <v>1.269987525779274</v>
+        <v>1.09849375521417</v>
       </c>
     </row>
     <row r="107">
@@ -37856,17 +37858,17 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:21</t>
+          <t>2026-10-19 21:35:17</t>
         </is>
       </c>
       <c r="D107" t="b">
         <v>0</v>
       </c>
       <c r="E107" t="n">
-        <v>1.154061465322902</v>
+        <v>0.9691806509902189</v>
       </c>
       <c r="F107" t="n">
-        <v>1.088230071141723</v>
+        <v>1.051757717078652</v>
       </c>
     </row>
     <row r="108">
@@ -37882,17 +37884,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:28</t>
+          <t>2026-10-19 21:35:29</t>
         </is>
       </c>
       <c r="D108" t="b">
         <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>1.319491464490042</v>
+        <v>0.9886227231843978</v>
       </c>
       <c r="F108" t="n">
-        <v>1.312891507320068</v>
+        <v>1.087749878502632</v>
       </c>
     </row>
     <row r="109">
@@ -37908,17 +37910,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:35</t>
+          <t>2026-10-19 21:35:43</t>
         </is>
       </c>
       <c r="D109" t="b">
         <v>0</v>
       </c>
       <c r="E109" t="n">
-        <v>1.177693707671259</v>
+        <v>0.9369373346460137</v>
       </c>
       <c r="F109" t="n">
-        <v>1.050747242268714</v>
+        <v>1.035145839479584</v>
       </c>
     </row>
     <row r="110">
@@ -37934,17 +37936,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:44</t>
+          <t>2026-10-19 21:35:55</t>
         </is>
       </c>
       <c r="D110" t="b">
         <v>1</v>
       </c>
       <c r="E110" t="n">
-        <v>1.325945408280003</v>
+        <v>1.030507166718694</v>
       </c>
       <c r="F110" t="n">
-        <v>1.317227609173262</v>
+        <v>1.123424448845442</v>
       </c>
     </row>
     <row r="111">
@@ -37960,17 +37962,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:53</t>
+          <t>2026-10-19 21:36:10</t>
         </is>
       </c>
       <c r="D111" t="b">
         <v>0</v>
       </c>
       <c r="E111" t="n">
-        <v>1.18871274720919</v>
+        <v>0.986389435341711</v>
       </c>
       <c r="F111" t="n">
-        <v>1.088230071141723</v>
+        <v>1.072043090896081</v>
       </c>
     </row>
     <row r="112">
@@ -37986,17 +37988,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2026-06-30 11:14:59</t>
+          <t>2026-10-19 21:36:22</t>
         </is>
       </c>
       <c r="D112" t="b">
         <v>1</v>
       </c>
       <c r="E112" t="n">
-        <v>0.7177673050417738</v>
+        <v>0.8370962261797386</v>
       </c>
       <c r="F112" t="n">
-        <v>0.7549455776854284</v>
+        <v>0.9309566361540316</v>
       </c>
     </row>
     <row r="113">
@@ -38012,17 +38014,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:09</t>
+          <t>2026-10-19 21:36:37</t>
         </is>
       </c>
       <c r="D113" t="b">
         <v>0</v>
       </c>
       <c r="E113" t="n">
-        <v>0.7401043976662182</v>
+        <v>0.8157669866399141</v>
       </c>
       <c r="F113" t="n">
-        <v>0.7153642844902806</v>
+        <v>0.8951889572250966</v>
       </c>
     </row>
     <row r="114">
@@ -38038,17 +38040,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:15</t>
+          <t>2026-10-19 21:36:49</t>
         </is>
       </c>
       <c r="D114" t="b">
         <v>1</v>
       </c>
       <c r="E114" t="n">
-        <v>0.7412066977460062</v>
+        <v>0.8671557263244883</v>
       </c>
       <c r="F114" t="n">
-        <v>0.7702574155321058</v>
+        <v>0.962236438134039</v>
       </c>
     </row>
     <row r="115">
@@ -38064,17 +38066,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:29</t>
+          <t>2026-10-19 21:37:03</t>
         </is>
       </c>
       <c r="D115" t="b">
         <v>0</v>
       </c>
       <c r="E115" t="n">
-        <v>0.7732948976612537</v>
+        <v>0.8501689247975242</v>
       </c>
       <c r="F115" t="n">
-        <v>0.730784994284864</v>
+        <v>0.9279160034267279</v>
       </c>
     </row>
     <row r="116">
@@ -38090,17 +38092,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:35</t>
+          <t>2026-10-19 21:37:14</t>
         </is>
       </c>
       <c r="D116" t="b">
         <v>1</v>
       </c>
       <c r="E116" t="n">
-        <v>0.7216673762260467</v>
+        <v>0.8431580813480345</v>
       </c>
       <c r="F116" t="n">
-        <v>0.7618607525791475</v>
+        <v>0.937429704138899</v>
       </c>
     </row>
     <row r="117">
@@ -38116,17 +38118,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:45</t>
+          <t>2026-10-19 21:37:28</t>
         </is>
       </c>
       <c r="D117" t="b">
         <v>0</v>
       </c>
       <c r="E117" t="n">
-        <v>0.7443821338491261</v>
+        <v>0.820873426669382</v>
       </c>
       <c r="F117" t="n">
-        <v>0.7205996104905891</v>
+        <v>0.9006344496763495</v>
       </c>
     </row>
     <row r="118">
@@ -38142,17 +38144,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2026-06-30 11:15:51</t>
+          <t>2026-10-19 21:37:39</t>
         </is>
       </c>
       <c r="D118" t="b">
         <v>1</v>
       </c>
       <c r="E118" t="n">
-        <v>0.7452761848234843</v>
+        <v>0.8732262787791567</v>
       </c>
       <c r="F118" t="n">
-        <v>0.7772355994200966</v>
+        <v>0.9689928491689139</v>
       </c>
     </row>
     <row r="119">
@@ -38168,17 +38170,17 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:06</t>
+          <t>2026-10-19 21:37:56</t>
         </is>
       </c>
       <c r="D119" t="b">
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0.7777560338726198</v>
+        <v>0.8557023325734013</v>
       </c>
       <c r="F119" t="n">
-        <v>0.7360882886945115</v>
+        <v>0.9334815476783511</v>
       </c>
     </row>
     <row r="120">
@@ -38194,17 +38196,17 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:16</t>
+          <t>2026-10-19 21:38:09</t>
         </is>
       </c>
       <c r="D120" t="b">
         <v>1</v>
       </c>
       <c r="E120" t="n">
-        <v>0.695694984344375</v>
+        <v>0.7952929006607702</v>
       </c>
       <c r="F120" t="n">
-        <v>0.7075509174749333</v>
+        <v>0.8862587607675692</v>
       </c>
     </row>
     <row r="121">
@@ -38220,17 +38222,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:25</t>
+          <t>2026-10-19 21:38:25</t>
         </is>
       </c>
       <c r="D121" t="b">
         <v>0</v>
       </c>
       <c r="E121" t="n">
-        <v>0.7332537560072732</v>
+        <v>0.7845731326383251</v>
       </c>
       <c r="F121" t="n">
-        <v>0.6790719569510054</v>
+        <v>0.8573018466553385</v>
       </c>
     </row>
     <row r="122">
@@ -38246,17 +38248,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:31</t>
+          <t>2026-10-19 21:38:35</t>
         </is>
       </c>
       <c r="D122" t="b">
         <v>1</v>
       </c>
       <c r="E122" t="n">
-        <v>0.7158439303628452</v>
+        <v>0.8244254732791108</v>
       </c>
       <c r="F122" t="n">
-        <v>0.7224237113213305</v>
+        <v>0.9167621736615972</v>
       </c>
     </row>
     <row r="123">
@@ -38272,17 +38274,17 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:38</t>
+          <t>2026-10-19 21:38:48</t>
         </is>
       </c>
       <c r="D123" t="b">
         <v>0</v>
       </c>
       <c r="E123" t="n">
-        <v>0.7954147799401795</v>
+        <v>0.8107815577362778</v>
       </c>
       <c r="F123" t="n">
-        <v>0.6940209028925668</v>
+        <v>0.8892007087882449</v>
       </c>
     </row>
     <row r="124">
@@ -38298,17 +38300,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:44</t>
+          <t>2026-10-19 21:39:02</t>
         </is>
       </c>
       <c r="D124" t="b">
         <v>1</v>
       </c>
       <c r="E124" t="n">
-        <v>0.9983676297386583</v>
+        <v>0.8143082167339285</v>
       </c>
       <c r="F124" t="n">
-        <v>0.9974632574897072</v>
+        <v>0.9059888346262379</v>
       </c>
     </row>
     <row r="125">
@@ -38324,17 +38326,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:51</t>
+          <t>2026-10-19 21:39:19</t>
         </is>
       </c>
       <c r="D125" t="b">
         <v>0</v>
       </c>
       <c r="E125" t="n">
-        <v>0.9277606238317307</v>
+        <v>0.7967008798725779</v>
       </c>
       <c r="F125" t="n">
-        <v>0.9474608642071516</v>
+        <v>0.8741706475626597</v>
       </c>
     </row>
     <row r="126">
@@ -38350,17 +38352,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2026-06-30 11:16:58</t>
+          <t>2026-10-19 21:39:32</t>
         </is>
       </c>
       <c r="D126" t="b">
         <v>1</v>
       </c>
       <c r="E126" t="n">
-        <v>1.008425118689472</v>
+        <v>0.8442121758618309</v>
       </c>
       <c r="F126" t="n">
-        <v>1.012801833586609</v>
+        <v>0.9367486281159833</v>
       </c>
     </row>
     <row r="127">
@@ -38376,17 +38378,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:07</t>
+          <t>2026-10-19 21:39:46</t>
         </is>
       </c>
       <c r="D127" t="b">
         <v>0</v>
       </c>
       <c r="E127" t="n">
-        <v>0.9267838015340176</v>
+        <v>0.8295317493985302</v>
       </c>
       <c r="F127" t="n">
-        <v>0.9799564785299339</v>
+        <v>0.9063700853852672</v>
       </c>
     </row>
     <row r="128">
@@ -38402,17 +38404,17 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:14</t>
+          <t>2026-10-19 21:39:57</t>
         </is>
       </c>
       <c r="D128" t="b">
         <v>1</v>
       </c>
       <c r="E128" t="n">
-        <v>1.033845692266929</v>
+        <v>0.8314859112133302</v>
       </c>
       <c r="F128" t="n">
-        <v>1.037117535362593</v>
+        <v>0.9243145795792789</v>
       </c>
     </row>
     <row r="129">
@@ -38428,17 +38430,17 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:23</t>
+          <t>2026-10-19 21:40:10</t>
         </is>
       </c>
       <c r="D129" t="b">
         <v>0</v>
       </c>
       <c r="E129" t="n">
-        <v>0.9673110888930337</v>
+        <v>0.8134738214776254</v>
       </c>
       <c r="F129" t="n">
-        <v>0.9474608642071516</v>
+        <v>0.8896776854844552</v>
       </c>
     </row>
     <row r="130">
@@ -38454,17 +38456,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:28</t>
+          <t>2026-10-19 21:40:20</t>
         </is>
       </c>
       <c r="D130" t="b">
         <v>1</v>
       </c>
       <c r="E130" t="n">
-        <v>1.043084646537483</v>
+        <v>0.8614172908837313</v>
       </c>
       <c r="F130" t="n">
-        <v>1.052456249952057</v>
+        <v>0.9553978727695803</v>
       </c>
     </row>
     <row r="131">
@@ -38480,17 +38482,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:36</t>
+          <t>2026-10-19 21:40:33</t>
         </is>
       </c>
       <c r="D131" t="b">
         <v>0</v>
       </c>
       <c r="E131" t="n">
-        <v>0.9643442792263704</v>
+        <v>0.8451187754494781</v>
       </c>
       <c r="F131" t="n">
-        <v>0.9799564785299339</v>
+        <v>0.9222128640219787</v>
       </c>
     </row>
     <row r="132">
@@ -38506,17 +38508,17 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:42</t>
+          <t>2026-10-19 21:40:44</t>
         </is>
       </c>
       <c r="D132" t="b">
         <v>1</v>
       </c>
       <c r="E132" t="n">
-        <v>1.256510542780482</v>
+        <v>0.9414931297837785</v>
       </c>
       <c r="F132" t="n">
-        <v>1.257826861978685</v>
+        <v>1.041147404943059</v>
       </c>
     </row>
     <row r="133">
@@ -38532,17 +38534,17 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:50</t>
+          <t>2026-10-19 21:40:57</t>
         </is>
       </c>
       <c r="D133" t="b">
         <v>0</v>
       </c>
       <c r="E133" t="n">
-        <v>1.135613661940718</v>
+        <v>0.8941714880970193</v>
       </c>
       <c r="F133" t="n">
-        <v>0.9474608642071516</v>
+        <v>0.9870125251589905</v>
       </c>
     </row>
     <row r="134">
@@ -38558,17 +38560,17 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2026-06-30 11:17:57</t>
+          <t>2026-10-19 21:41:08</t>
         </is>
       </c>
       <c r="D134" t="b">
         <v>1</v>
       </c>
       <c r="E134" t="n">
-        <v>1.264650053304709</v>
+        <v>0.9805220116680951</v>
       </c>
       <c r="F134" t="n">
-        <v>1.261927513437551</v>
+        <v>1.073896912975074</v>
       </c>
     </row>
     <row r="135">
@@ -38584,17 +38586,17 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:06</t>
+          <t>2026-10-19 21:41:21</t>
         </is>
       </c>
       <c r="D135" t="b">
         <v>0</v>
       </c>
       <c r="E135" t="n">
-        <v>1.139214358124869</v>
+        <v>0.9385074100205172</v>
       </c>
       <c r="F135" t="n">
-        <v>0.9799564785299339</v>
+        <v>1.020960254468962</v>
       </c>
     </row>
     <row r="136">
@@ -38610,17 +38612,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:12</t>
+          <t>2026-10-19 21:41:32</t>
         </is>
       </c>
       <c r="D136" t="b">
         <v>1</v>
       </c>
       <c r="E136" t="n">
-        <v>1.310498784520148</v>
+        <v>0.9634527977452739</v>
       </c>
       <c r="F136" t="n">
-        <v>1.305061260468013</v>
+        <v>1.065129524247215</v>
       </c>
     </row>
     <row r="137">
@@ -38636,17 +38638,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:21</t>
+          <t>2026-10-19 21:41:47</t>
         </is>
       </c>
       <c r="D137" t="b">
         <v>0</v>
       </c>
       <c r="E137" t="n">
-        <v>1.163223062173153</v>
+        <v>0.9098270335935762</v>
       </c>
       <c r="F137" t="n">
-        <v>0.9474608642071516</v>
+        <v>1.005173149600356</v>
       </c>
     </row>
     <row r="138">
@@ -38662,17 +38664,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:26</t>
+          <t>2026-10-19 21:41:58</t>
         </is>
       </c>
       <c r="D138" t="b">
         <v>1</v>
       </c>
       <c r="E138" t="n">
-        <v>1.317209476166313</v>
+        <v>1.00295709008329</v>
       </c>
       <c r="F138" t="n">
-        <v>1.309163850811504</v>
+        <v>1.098505410039371</v>
       </c>
     </row>
     <row r="139">
@@ -38688,17 +38690,17 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:34</t>
+          <t>2026-10-19 21:42:11</t>
         </is>
       </c>
       <c r="D139" t="b">
         <v>0</v>
       </c>
       <c r="E139" t="n">
-        <v>1.174683750810882</v>
+        <v>0.9557604129001379</v>
       </c>
       <c r="F139" t="n">
-        <v>0.9799564785299339</v>
+        <v>1.041216562750644</v>
       </c>
     </row>
     <row r="140">
@@ -38714,17 +38716,17 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:44</t>
+          <t>2026-10-19 21:42:21</t>
         </is>
       </c>
       <c r="D140" t="b">
         <v>1</v>
       </c>
       <c r="E140" t="n">
-        <v>0.7422358954785195</v>
+        <v>0.8630196083632683</v>
       </c>
       <c r="F140" t="n">
-        <v>0.7697005745018751</v>
+        <v>0.9551624601118291</v>
       </c>
     </row>
     <row r="141">
@@ -38740,17 +38742,17 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>2026-06-30 11:18:57</t>
+          <t>2026-10-19 21:42:36</t>
         </is>
       </c>
       <c r="D141" t="b">
         <v>0</v>
       </c>
       <c r="E141" t="n">
-        <v>0.7666128071678421</v>
+        <v>0.8426316458595161</v>
       </c>
       <c r="F141" t="n">
-        <v>0.7318533549630347</v>
+        <v>0.9252373288486294</v>
       </c>
     </row>
     <row r="142">
@@ -38766,17 +38768,17 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:02</t>
+          <t>2026-10-19 21:42:47</t>
         </is>
       </c>
       <c r="D142" t="b">
         <v>1</v>
       </c>
       <c r="E142" t="n">
-        <v>0.7605729688136886</v>
+        <v>0.8946724187825181</v>
       </c>
       <c r="F142" t="n">
-        <v>0.7862759896519566</v>
+        <v>0.9886307627851824</v>
       </c>
     </row>
     <row r="143">
@@ -38792,17 +38794,17 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:10</t>
+          <t>2026-10-19 21:43:00</t>
         </is>
       </c>
       <c r="D143" t="b">
         <v>0</v>
       </c>
       <c r="E143" t="n">
-        <v>0.7977655216983451</v>
+        <v>0.879328461424298</v>
       </c>
       <c r="F143" t="n">
-        <v>0.7488161855827953</v>
+        <v>0.9599745047875515</v>
       </c>
     </row>
     <row r="144">
@@ -38818,17 +38820,17 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:20</t>
+          <t>2026-10-19 21:43:10</t>
         </is>
       </c>
       <c r="D144" t="b">
         <v>1</v>
       </c>
       <c r="E144" t="n">
-        <v>0.7463066896815055</v>
+        <v>0.8693025851104071</v>
       </c>
       <c r="F144" t="n">
-        <v>0.776676478084194</v>
+        <v>0.9617229489117616</v>
       </c>
     </row>
     <row r="145">
@@ -38844,17 +38846,17 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:33</t>
+          <t>2026-10-19 21:43:24</t>
         </is>
       </c>
       <c r="D145" t="b">
         <v>0</v>
       </c>
       <c r="E145" t="n">
-        <v>0.7632242539039238</v>
+        <v>0.8476881183403533</v>
       </c>
       <c r="F145" t="n">
-        <v>0.7371613322429842</v>
+        <v>0.9307931401470877</v>
       </c>
     </row>
     <row r="146">
@@ -38870,17 +38872,17 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:39</t>
+          <t>2026-10-19 21:43:38</t>
         </is>
       </c>
       <c r="D146" t="b">
         <v>1</v>
       </c>
       <c r="E146" t="n">
-        <v>0.7647193909130752</v>
+        <v>0.9007150775207181</v>
       </c>
       <c r="F146" t="n">
-        <v>0.7933194072139826</v>
+        <v>0.9954096393065119</v>
       </c>
     </row>
     <row r="147">
@@ -38896,17 +38898,17 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2026-06-30 11:19:52</t>
+          <t>2026-10-19 21:43:54</t>
         </is>
       </c>
       <c r="D147" t="b">
         <v>0</v>
       </c>
       <c r="E147" t="n">
-        <v>0.8021012679266721</v>
+        <v>0.8850889857885215</v>
       </c>
       <c r="F147" t="n">
-        <v>0.7541980604135141</v>
+        <v>0.9656552496874866</v>
       </c>
     </row>
     <row r="148">
@@ -38922,17 +38924,17 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:02</t>
+          <t>2026-10-19 21:44:05</t>
         </is>
       </c>
       <c r="D148" t="b">
         <v>1</v>
       </c>
       <c r="E148" t="n">
-        <v>0.7137163659457456</v>
+        <v>0.8197542774068484</v>
       </c>
       <c r="F148" t="n">
-        <v>0.721882752756499</v>
+        <v>0.909862150817111</v>
       </c>
     </row>
     <row r="149">
@@ -38948,17 +38950,17 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:10</t>
+          <t>2026-10-19 21:44:19</t>
         </is>
       </c>
       <c r="D149" t="b">
         <v>0</v>
       </c>
       <c r="E149" t="n">
-        <v>0.7637299558543261</v>
+        <v>0.805259170539687</v>
       </c>
       <c r="F149" t="n">
-        <v>0.6946303967823044</v>
+        <v>0.8865891405602859</v>
       </c>
     </row>
     <row r="150">
@@ -38974,17 +38976,17 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:16</t>
+          <t>2026-10-19 21:44:29</t>
         </is>
       </c>
       <c r="D150" t="b">
         <v>1</v>
       </c>
       <c r="E150" t="n">
-        <v>0.7317067589650644</v>
+        <v>0.8497038956052918</v>
       </c>
       <c r="F150" t="n">
-        <v>0.7379881353134501</v>
+        <v>0.9365999452657284</v>
       </c>
     </row>
     <row r="151">
@@ -39000,17 +39002,17 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:24</t>
+          <t>2026-10-19 21:44:41</t>
         </is>
       </c>
       <c r="D151" t="b">
         <v>0</v>
       </c>
       <c r="E151" t="n">
-        <v>0.8222649664599543</v>
+        <v>0.8384755958285527</v>
       </c>
       <c r="F151" t="n">
-        <v>0.7114539802840065</v>
+        <v>0.9204654144128032</v>
       </c>
     </row>
     <row r="152">
@@ -39026,17 +39028,17 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:30</t>
+          <t>2026-10-19 21:44:51</t>
         </is>
       </c>
       <c r="D152" t="b">
         <v>1</v>
       </c>
       <c r="E152" t="n">
-        <v>1.007844042742936</v>
+        <v>0.8361100951622745</v>
       </c>
       <c r="F152" t="n">
-        <v>1.010889037657477</v>
+        <v>0.929791181771104</v>
       </c>
     </row>
     <row r="153">
@@ -39052,17 +39054,17 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:38</t>
+          <t>2026-10-19 21:45:05</t>
         </is>
       </c>
       <c r="D153" t="b">
         <v>0</v>
       </c>
       <c r="E153" t="n">
-        <v>0.9297371401515656</v>
+        <v>0.8284783796143715</v>
       </c>
       <c r="F153" t="n">
-        <v>1.010889037657477</v>
+        <v>0.9037341346269492</v>
       </c>
     </row>
     <row r="154">
@@ -39078,17 +39080,17 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:44</t>
+          <t>2026-10-19 21:45:15</t>
         </is>
       </c>
       <c r="D154" t="b">
         <v>1</v>
       </c>
       <c r="E154" t="n">
-        <v>1.023665699022344</v>
+        <v>0.8720879956747716</v>
       </c>
       <c r="F154" t="n">
-        <v>1.027516549861404</v>
+        <v>0.9627970294167952</v>
       </c>
     </row>
     <row r="155">
@@ -39104,17 +39106,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:52</t>
+          <t>2026-10-19 21:45:27</t>
         </is>
       </c>
       <c r="D155" t="b">
         <v>0</v>
       </c>
       <c r="E155" t="n">
-        <v>0.9543627090166708</v>
+        <v>0.8577495573022746</v>
       </c>
       <c r="F155" t="n">
-        <v>1.027516549861404</v>
+        <v>0.9379213207049641</v>
       </c>
     </row>
     <row r="156">
@@ -39130,17 +39132,17 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-06-30 11:20:58</t>
+          <t>2026-10-19 21:45:38</t>
         </is>
       </c>
       <c r="D156" t="b">
         <v>1</v>
       </c>
       <c r="E156" t="n">
-        <v>1.043176340088655</v>
+        <v>0.8571799415904316</v>
       </c>
       <c r="F156" t="n">
-        <v>1.050543437095388</v>
+        <v>0.9483678512838237</v>
       </c>
     </row>
     <row r="157">
@@ -39156,17 +39158,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:07</t>
+          <t>2026-10-19 21:45:51</t>
         </is>
       </c>
       <c r="D157" t="b">
         <v>0</v>
       </c>
       <c r="E157" t="n">
-        <v>0.9696459170793412</v>
+        <v>0.8378843637043218</v>
       </c>
       <c r="F157" t="n">
-        <v>1.049257007431511</v>
+        <v>0.9195497602306472</v>
       </c>
     </row>
     <row r="158">
@@ -39182,17 +39184,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:13</t>
+          <t>2026-10-19 21:46:01</t>
         </is>
       </c>
       <c r="D158" t="b">
         <v>1</v>
       </c>
       <c r="E158" t="n">
-        <v>1.058515232149438</v>
+        <v>0.8888020279778518</v>
       </c>
       <c r="F158" t="n">
-        <v>1.06717109330398</v>
+        <v>0.9816501548573658</v>
       </c>
     </row>
     <row r="159">
@@ -39208,17 +39210,17 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:23</t>
+          <t>2026-10-19 21:46:13</t>
         </is>
       </c>
       <c r="D159" t="b">
         <v>0</v>
       </c>
       <c r="E159" t="n">
-        <v>0.9832128965414374</v>
+        <v>0.8744785131540802</v>
       </c>
       <c r="F159" t="n">
-        <v>1.053492157466119</v>
+        <v>0.9540867650034452</v>
       </c>
     </row>
     <row r="160">
@@ -39234,17 +39236,17 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:30</t>
+          <t>2026-10-19 21:46:23</t>
         </is>
       </c>
       <c r="D160" t="b">
         <v>1</v>
       </c>
       <c r="E160" t="n">
-        <v>1.267042161092413</v>
+        <v>0.9693179165031311</v>
       </c>
       <c r="F160" t="n">
-        <v>1.267288204185221</v>
+        <v>1.066492658620385</v>
       </c>
     </row>
     <row r="161">
@@ -39260,17 +39262,17 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:38</t>
+          <t>2026-10-19 21:46:36</t>
         </is>
       </c>
       <c r="D161" t="b">
         <v>0</v>
       </c>
       <c r="E161" t="n">
-        <v>1.141632809605668</v>
+        <v>0.9254006672967249</v>
       </c>
       <c r="F161" t="n">
-        <v>1.055328404038741</v>
+        <v>1.018173979328351</v>
       </c>
     </row>
     <row r="162">
@@ -39286,17 +39288,17 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:44</t>
+          <t>2026-10-19 21:46:46</t>
         </is>
       </c>
       <c r="D162" t="b">
         <v>1</v>
       </c>
       <c r="E162" t="n">
-        <v>1.276602039124883</v>
+        <v>1.010552395130111</v>
       </c>
       <c r="F162" t="n">
-        <v>1.271622376211204</v>
+        <v>1.101454363286823</v>
       </c>
     </row>
     <row r="163">
@@ -39312,17 +39314,17 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:52</t>
+          <t>2026-10-19 21:47:01</t>
         </is>
       </c>
       <c r="D163" t="b">
         <v>0</v>
       </c>
       <c r="E163" t="n">
-        <v>1.155991342863616</v>
+        <v>0.9704769263443318</v>
       </c>
       <c r="F163" t="n">
-        <v>1.093726180937058</v>
+        <v>1.05487945320136</v>
       </c>
     </row>
     <row r="164">
@@ -39338,17 +39340,17 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2026-06-30 11:21:58</t>
+          <t>2026-10-19 21:47:11</t>
         </is>
       </c>
       <c r="D164" t="b">
         <v>1</v>
       </c>
       <c r="E164" t="n">
-        <v>1.321425801722621</v>
+        <v>0.9917432901290253</v>
       </c>
       <c r="F164" t="n">
-        <v>1.314527042502297</v>
+        <v>1.090773562218706</v>
       </c>
     </row>
     <row r="165">
@@ -39364,17 +39366,17 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:07</t>
+          <t>2026-10-19 21:47:24</t>
         </is>
       </c>
       <c r="D165" t="b">
         <v>0</v>
       </c>
       <c r="E165" t="n">
-        <v>1.17952129404422</v>
+        <v>0.940260522562319</v>
       </c>
       <c r="F165" t="n">
-        <v>1.055328404038741</v>
+        <v>1.038354890421243</v>
       </c>
     </row>
     <row r="166">
@@ -39390,17 +39392,17 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:15</t>
+          <t>2026-10-19 21:47:34</t>
         </is>
       </c>
       <c r="D166" t="b">
         <v>1</v>
       </c>
       <c r="E166" t="n">
-        <v>1.327868803199202</v>
+        <v>1.033632328042161</v>
       </c>
       <c r="F166" t="n">
-        <v>1.318863209103888</v>
+        <v>1.126423124662476</v>
       </c>
     </row>
     <row r="167">
@@ -39416,17 +39418,17 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:23</t>
+          <t>2026-10-19 21:47:47</t>
         </is>
       </c>
       <c r="D167" t="b">
         <v>0</v>
       </c>
       <c r="E167" t="n">
-        <v>1.190537856705349</v>
+        <v>0.9896259644350566</v>
       </c>
       <c r="F167" t="n">
-        <v>1.093726180937058</v>
+        <v>1.075195329204232</v>
       </c>
     </row>
     <row r="168">
@@ -39442,17 +39444,17 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:29</t>
+          <t>2026-10-19 21:47:58</t>
         </is>
       </c>
       <c r="D168" t="b">
         <v>1</v>
       </c>
       <c r="E168" t="n">
-        <v>0.7202637029065388</v>
+        <v>0.8400780724837894</v>
       </c>
       <c r="F168" t="n">
-        <v>0.7574287861669978</v>
+        <v>0.9338286181164154</v>
       </c>
     </row>
     <row r="169">
@@ -39468,17 +39470,17 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:40</t>
+          <t>2026-10-19 21:48:11</t>
         </is>
       </c>
       <c r="D169" t="b">
         <v>0</v>
       </c>
       <c r="E169" t="n">
-        <v>0.7425752586744948</v>
+        <v>0.818834108200402</v>
       </c>
       <c r="F169" t="n">
-        <v>0.7180399473856598</v>
+        <v>0.8982111179314876</v>
       </c>
     </row>
     <row r="170">
@@ -39494,17 +39496,17 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:46</t>
+          <t>2026-10-19 21:48:21</t>
         </is>
       </c>
       <c r="D170" t="b">
         <v>1</v>
       </c>
       <c r="E170" t="n">
-        <v>0.743682231215819</v>
+        <v>0.8700896043424849</v>
       </c>
       <c r="F170" t="n">
-        <v>0.7727223166292857</v>
+        <v>0.9652649643759439</v>
       </c>
     </row>
     <row r="171">
@@ -39520,17 +39522,17 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>2026-06-30 11:22:59</t>
+          <t>2026-10-19 21:48:34</t>
         </is>
       </c>
       <c r="D171" t="b">
         <v>0</v>
       </c>
       <c r="E171" t="n">
-        <v>0.7757547748067121</v>
+        <v>0.8532632055159782</v>
       </c>
       <c r="F171" t="n">
-        <v>0.7334414544445873</v>
+        <v>0.9309106048347273</v>
       </c>
     </row>
     <row r="172">
@@ -39546,17 +39548,17 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:05</t>
+          <t>2026-10-19 21:48:49</t>
         </is>
       </c>
       <c r="D172" t="b">
         <v>1</v>
       </c>
       <c r="E172" t="n">
-        <v>0.7241739843458126</v>
+        <v>0.8461516661395417</v>
       </c>
       <c r="F172" t="n">
-        <v>0.7643542225019402</v>
+        <v>0.9403121389304249</v>
       </c>
     </row>
     <row r="173">
@@ -39572,17 +39574,17 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:14</t>
+          <t>2026-10-19 21:49:04</t>
         </is>
       </c>
       <c r="D173" t="b">
         <v>0</v>
       </c>
       <c r="E173" t="n">
-        <v>0.7468588933591208</v>
+        <v>0.8239525710856679</v>
       </c>
       <c r="F173" t="n">
-        <v>0.7232871169389228</v>
+        <v>0.9036678005112359</v>
       </c>
     </row>
     <row r="174">
@@ -39598,17 +39600,17 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:20</t>
+          <t>2026-10-19 21:49:16</t>
         </is>
       </c>
       <c r="D174" t="b">
         <v>1</v>
       </c>
       <c r="E174" t="n">
-        <v>0.7477614039435903</v>
+        <v>0.8761697542295133</v>
       </c>
       <c r="F174" t="n">
-        <v>0.7797105843184732</v>
+        <v>0.9718338840433846</v>
       </c>
     </row>
     <row r="175">
@@ -39624,17 +39626,17 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:33</t>
+          <t>2026-10-19 21:49:30</t>
         </is>
       </c>
       <c r="D175" t="b">
         <v>0</v>
       </c>
       <c r="E175" t="n">
-        <v>0.7802232809677351</v>
+        <v>0.85880969323345</v>
       </c>
       <c r="F175" t="n">
-        <v>0.738756386474117</v>
+        <v>0.9364870103303705</v>
       </c>
     </row>
     <row r="176">
@@ -39650,17 +39652,17 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:42</t>
+          <t>2026-10-19 21:49:41</t>
         </is>
       </c>
       <c r="D176" t="b">
         <v>1</v>
       </c>
       <c r="E176" t="n">
-        <v>0.6981258319694563</v>
+        <v>0.7982007300022034</v>
       </c>
       <c r="F176" t="n">
-        <v>0.7099625986510174</v>
+        <v>0.8890586794745517</v>
       </c>
     </row>
     <row r="177">
@@ -39676,17 +39678,17 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:50</t>
+          <t>2026-10-19 21:49:57</t>
         </is>
       </c>
       <c r="D177" t="b">
         <v>0</v>
       </c>
       <c r="E177" t="n">
-        <v>0.7347065977592583</v>
+        <v>0.7875490549328629</v>
       </c>
       <c r="F177" t="n">
-        <v>0.6816653904037245</v>
+        <v>0.8602467692879511</v>
       </c>
     </row>
     <row r="178">
@@ -39702,17 +39704,17 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2026-06-30 11:23:55</t>
+          <t>2026-10-19 21:50:09</t>
         </is>
       </c>
       <c r="D178" t="b">
         <v>1</v>
       </c>
       <c r="E178" t="n">
-        <v>0.7182607308210408</v>
+        <v>0.8272918704135929</v>
       </c>
       <c r="F178" t="n">
-        <v>0.724818384026505</v>
+        <v>0.9195400804340638</v>
       </c>
     </row>
     <row r="179">
@@ -39728,17 +39730,17 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:03</t>
+          <t>2026-10-19 21:50:23</t>
         </is>
       </c>
       <c r="D179" t="b">
         <v>0</v>
       </c>
       <c r="E179" t="n">
-        <v>0.7980167736586693</v>
+        <v>0.8137910754236982</v>
       </c>
       <c r="F179" t="n">
-        <v>0.6965966205679841</v>
+        <v>0.8921204321615087</v>
       </c>
     </row>
     <row r="180">
@@ -39754,17 +39756,17 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:09</t>
+          <t>2026-10-19 21:50:34</t>
         </is>
       </c>
       <c r="D180" t="b">
         <v>1</v>
       </c>
       <c r="E180" t="n">
-        <v>1.000295603679186</v>
+        <v>0.8172389684666425</v>
       </c>
       <c r="F180" t="n">
-        <v>0.9992874272229116</v>
+        <v>0.9088129115909777</v>
       </c>
     </row>
     <row r="181">
@@ -39780,17 +39782,17 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:18</t>
+          <t>2026-10-19 21:50:52</t>
         </is>
       </c>
       <c r="D181" t="b">
         <v>0</v>
       </c>
       <c r="E181" t="n">
-        <v>0.9295458421217276</v>
+        <v>0.7997871719114513</v>
       </c>
       <c r="F181" t="n">
-        <v>0.9513091299213262</v>
+        <v>0.8771435651747608</v>
       </c>
     </row>
     <row r="182">
@@ -39806,17 +39808,17 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:24</t>
+          <t>2026-10-19 21:51:03</t>
         </is>
       </c>
       <c r="D182" t="b">
         <v>1</v>
       </c>
       <c r="E182" t="n">
-        <v>1.010366213463529</v>
+        <v>0.8470917570924951</v>
       </c>
       <c r="F182" t="n">
-        <v>1.014626095885179</v>
+        <v>0.9395495756862482</v>
       </c>
     </row>
     <row r="183">
@@ -39832,17 +39834,17 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:32</t>
+          <t>2026-10-19 21:51:18</t>
         </is>
       </c>
       <c r="D183" t="b">
         <v>0</v>
       </c>
       <c r="E183" t="n">
-        <v>0.9286358545376127</v>
+        <v>0.8322196100820758</v>
       </c>
       <c r="F183" t="n">
-        <v>0.9845733133307029</v>
+        <v>0.9093170221598921</v>
       </c>
     </row>
     <row r="184">
@@ -39858,17 +39860,17 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:38</t>
+          <t>2026-10-19 21:51:29</t>
         </is>
       </c>
       <c r="D184" t="b">
         <v>1</v>
       </c>
       <c r="E184" t="n">
-        <v>1.035773655433925</v>
+        <v>0.8344501053289798</v>
       </c>
       <c r="F184" t="n">
-        <v>1.03894180772777</v>
+        <v>0.9271682835543118</v>
       </c>
     </row>
     <row r="185">
@@ -39884,17 +39886,17 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:45</t>
+          <t>2026-10-19 21:51:46</t>
         </is>
       </c>
       <c r="D185" t="b">
         <v>0</v>
       </c>
       <c r="E185" t="n">
-        <v>0.9691425382303854</v>
+        <v>0.8213295781859531</v>
       </c>
       <c r="F185" t="n">
-        <v>0.9513091299213262</v>
+        <v>0.8926819192656369</v>
       </c>
     </row>
     <row r="186">
@@ -39910,17 +39912,17 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:51</t>
+          <t>2026-10-19 21:51:57</t>
         </is>
       </c>
       <c r="D186" t="b">
         <v>1</v>
       </c>
       <c r="E186" t="n">
-        <v>1.045007897201579</v>
+        <v>0.8643362923590628</v>
       </c>
       <c r="F186" t="n">
-        <v>1.054280528305624</v>
+        <v>0.9582279051328597</v>
       </c>
     </row>
     <row r="187">
@@ -39936,17 +39938,17 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>2026-06-30 11:24:59</t>
+          <t>2026-10-19 21:52:10</t>
         </is>
       </c>
       <c r="D187" t="b">
         <v>0</v>
       </c>
       <c r="E187" t="n">
-        <v>0.9661295083855056</v>
+        <v>0.8482289636364775</v>
       </c>
       <c r="F187" t="n">
-        <v>0.9845733133307029</v>
+        <v>0.9251900133698469</v>
       </c>
     </row>
     <row r="188">
@@ -39962,17 +39964,17 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:05</t>
+          <t>2026-10-19 21:52:21</t>
         </is>
       </c>
       <c r="D188" t="b">
         <v>1</v>
       </c>
       <c r="E188" t="n">
-        <v>1.258444906474659</v>
+        <v>0.9448414452257936</v>
       </c>
       <c r="F188" t="n">
-        <v>1.259461502649863</v>
+        <v>1.044155326513956</v>
       </c>
     </row>
     <row r="189">
@@ -39988,17 +39990,17 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:14</t>
+          <t>2026-10-19 21:52:34</t>
         </is>
       </c>
       <c r="D189" t="b">
         <v>0</v>
       </c>
       <c r="E189" t="n">
-        <v>1.137561821224532</v>
+        <v>0.8970729324525337</v>
       </c>
       <c r="F189" t="n">
-        <v>0.9513091299213262</v>
+        <v>0.9901441553680648</v>
       </c>
     </row>
     <row r="190">
@@ -40014,17 +40016,17 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:20</t>
+          <t>2026-10-19 21:52:44</t>
         </is>
       </c>
       <c r="D190" t="b">
         <v>1</v>
       </c>
       <c r="E190" t="n">
-        <v>1.2665744878779</v>
+        <v>0.9840672940436507</v>
       </c>
       <c r="F190" t="n">
-        <v>1.263562225665089</v>
+        <v>1.076877186231826</v>
       </c>
     </row>
     <row r="191">
@@ -40040,17 +40042,17 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:32</t>
+          <t>2026-10-19 21:53:00</t>
         </is>
       </c>
       <c r="D191" t="b">
         <v>0</v>
       </c>
       <c r="E191" t="n">
-        <v>1.141144926253807</v>
+        <v>0.9418034747266891</v>
       </c>
       <c r="F191" t="n">
-        <v>0.9845733133307029</v>
+        <v>1.024338585343399</v>
       </c>
     </row>
     <row r="192">
@@ -40066,17 +40068,17 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:39</t>
+          <t>2026-10-19 21:53:13</t>
         </is>
       </c>
       <c r="D192" t="b">
         <v>1</v>
       </c>
       <c r="E192" t="n">
-        <v>1.312438239937259</v>
+        <v>0.9666636071597475</v>
       </c>
       <c r="F192" t="n">
-        <v>1.30669667674167</v>
+        <v>1.068173757361678</v>
       </c>
     </row>
     <row r="193">
@@ -40092,17 +40094,17 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:47</t>
+          <t>2026-10-19 21:53:27</t>
         </is>
       </c>
       <c r="D193" t="b">
         <v>0</v>
       </c>
       <c r="E193" t="n">
-        <v>1.165051147448593</v>
+        <v>0.9131778590275695</v>
       </c>
       <c r="F193" t="n">
-        <v>0.9513091299213262</v>
+        <v>1.00845070342817</v>
       </c>
     </row>
     <row r="194">
@@ -40118,17 +40120,17 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>2026-06-30 11:25:53</t>
+          <t>2026-10-19 21:53:39</t>
         </is>
       </c>
       <c r="D194" t="b">
         <v>1</v>
       </c>
       <c r="E194" t="n">
-        <v>1.319137727528867</v>
+        <v>1.006236904811878</v>
       </c>
       <c r="F194" t="n">
-        <v>1.310799329707921</v>
+        <v>1.101525301887871</v>
       </c>
     </row>
     <row r="195">
@@ -40144,17 +40146,17 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>2026-06-30 11:26:00</t>
+          <t>2026-10-19 21:53:53</t>
         </is>
       </c>
       <c r="D195" t="b">
         <v>0</v>
       </c>
       <c r="E195" t="n">
-        <v>1.176511336754921</v>
+        <v>0.9590901662555967</v>
       </c>
       <c r="F195" t="n">
-        <v>0.9845733133307029</v>
+        <v>1.044394673447659</v>
       </c>
     </row>
   </sheetData>

</xml_diff>